<commit_message>
Updated Case Manager Test Case
</commit_message>
<xml_diff>
--- a/test_data/Users_Test_Data.xlsx
+++ b/test_data/Users_Test_Data.xlsx
@@ -1,37 +1,101 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
-  <workbookProtection/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Rishi Files\OrthoLegal_Automation\test_data\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E63F9A0-2D96-4DFF-AA66-F5CB335E34A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="22932" yWindow="1092" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Users" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Users" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="15">
+  <si>
+    <t>Select Role</t>
+  </si>
+  <si>
+    <t>First Name</t>
+  </si>
+  <si>
+    <t>Middle Name</t>
+  </si>
+  <si>
+    <t>Last Name</t>
+  </si>
+  <si>
+    <t>Ortho Legal Email</t>
+  </si>
+  <si>
+    <t>Personal Email</t>
+  </si>
+  <si>
+    <t>Password</t>
+  </si>
+  <si>
+    <t>Confirm Password</t>
+  </si>
+  <si>
+    <t>Case Manager</t>
+  </si>
+  <si>
+    <t>Case</t>
+  </si>
+  <si>
+    <t>Manager</t>
+  </si>
+  <si>
+    <t>case.manager.sample@example.com</t>
+  </si>
+  <si>
+    <t>OrthoLegal@1234</t>
+  </si>
+  <si>
+    <t>Neoers</t>
+  </si>
+  <si>
+    <t>neoerscasemanager1@ortholegalgroup.com</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b val="1"/>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -46,85 +110,29 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+  <cellXfs count="3">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -412,109 +420,73 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:H2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="34" customWidth="1" min="5" max="5"/>
-    <col width="34" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
-    <col width="20" customWidth="1" min="8" max="8"/>
+    <col min="1" max="4" width="18" customWidth="1"/>
+    <col min="5" max="5" width="41.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="34" customWidth="1"/>
+    <col min="7" max="7" width="20" customWidth="1"/>
+    <col min="8" max="8" width="17.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Select Role</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>First Name</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Middle Name</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Last Name</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Ortho Legal Email</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Personal Email</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Password</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Confirm Password</t>
-        </is>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Case Manager</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Case</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Manager</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Sample</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>casemanager1@ortholegalgroup.com</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>case.manager.sample@example.com</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>OrthoLegal@1234</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>OrthoLegal@1234</t>
-        </is>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="F2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G2" t="s">
+        <v>12</v>
+      </c>
+      <c r="H2" t="s">
+        <v>12</v>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="E2" r:id="rId1" xr:uid="{24504C49-B5A8-4E23-8032-F4A43698753D}"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Corrected all Test Cases
</commit_message>
<xml_diff>
--- a/test_data/Users_Test_Data.xlsx
+++ b/test_data/Users_Test_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Rishi Files\OrthoLegal_Automation\test_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A108F97-BD31-4742-9EEB-8531758F280E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AAA8B030-389D-426E-B57E-3DA8A66F5AF3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="1092" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Users" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="51">
   <si>
     <t>Select Role</t>
   </si>
@@ -52,12 +52,6 @@
     <t>Neoers</t>
   </si>
   <si>
-    <t>Case</t>
-  </si>
-  <si>
-    <t>Manager</t>
-  </si>
-  <si>
     <t>neoerscasemanager1@ortholegalgroup.com</t>
   </si>
   <si>
@@ -94,30 +88,6 @@
     <t>Report Finalizer</t>
   </si>
   <si>
-    <t>Record</t>
-  </si>
-  <si>
-    <t>Medical</t>
-  </si>
-  <si>
-    <t>Report</t>
-  </si>
-  <si>
-    <t>Reviewer</t>
-  </si>
-  <si>
-    <t>Assistant</t>
-  </si>
-  <si>
-    <t>Finalizer</t>
-  </si>
-  <si>
-    <t>RecordReviewer</t>
-  </si>
-  <si>
-    <t>MedicalAssistant</t>
-  </si>
-  <si>
     <t>neoershistorian1@ortholegalgroup.com</t>
   </si>
   <si>
@@ -170,6 +140,39 @@
   </si>
   <si>
     <t>report.finalizer.sample@example.com</t>
+  </si>
+  <si>
+    <t>EditorA</t>
+  </si>
+  <si>
+    <t>HistorianA</t>
+  </si>
+  <si>
+    <t>HistorianManagerA</t>
+  </si>
+  <si>
+    <t>RecordReviewerManagerA</t>
+  </si>
+  <si>
+    <t>MedicalAssistantManagerA</t>
+  </si>
+  <si>
+    <t>EditorManagerA</t>
+  </si>
+  <si>
+    <t>Test</t>
+  </si>
+  <si>
+    <t>CaseManagerA</t>
+  </si>
+  <si>
+    <t>RecordReviewerA</t>
+  </si>
+  <si>
+    <t>MedicalAssistantA</t>
+  </si>
+  <si>
+    <t>ReportFinalizerA</t>
   </si>
 </sst>
 </file>
@@ -571,250 +574,256 @@
         <v>9</v>
       </c>
       <c r="C2" t="s">
+        <v>46</v>
+      </c>
+      <c r="D2" t="s">
+        <v>47</v>
+      </c>
+      <c r="E2" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="D2" t="s">
+      <c r="F2" t="s">
         <v>11</v>
       </c>
-      <c r="E2" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F2" t="s">
-        <v>13</v>
-      </c>
       <c r="G2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="H2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B3" t="s">
         <v>9</v>
       </c>
+      <c r="C3" t="s">
+        <v>46</v>
+      </c>
       <c r="D3" t="s">
-        <v>15</v>
+        <v>41</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>32</v>
+        <v>22</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>41</v>
+        <v>31</v>
       </c>
       <c r="G3" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="H3" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B4" t="s">
         <v>9</v>
       </c>
       <c r="C4" t="s">
-        <v>15</v>
+        <v>46</v>
       </c>
       <c r="D4" t="s">
-        <v>11</v>
+        <v>42</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>34</v>
+        <v>24</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>43</v>
+        <v>33</v>
       </c>
       <c r="G4" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="H4" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B5" t="s">
         <v>9</v>
       </c>
       <c r="C5" t="s">
-        <v>24</v>
+        <v>46</v>
       </c>
       <c r="D5" t="s">
-        <v>27</v>
+        <v>48</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>44</v>
+        <v>34</v>
       </c>
       <c r="G5" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="H5" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B6" t="s">
         <v>9</v>
       </c>
       <c r="C6" t="s">
-        <v>30</v>
+        <v>46</v>
       </c>
       <c r="D6" t="s">
-        <v>11</v>
+        <v>43</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>36</v>
+        <v>26</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>45</v>
+        <v>35</v>
       </c>
       <c r="G6" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="H6" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B7" t="s">
         <v>9</v>
       </c>
       <c r="C7" t="s">
-        <v>25</v>
+        <v>46</v>
       </c>
       <c r="D7" t="s">
-        <v>28</v>
+        <v>49</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>37</v>
+        <v>27</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>46</v>
+        <v>36</v>
       </c>
       <c r="G7" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="H7" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B8" t="s">
         <v>9</v>
       </c>
       <c r="C8" t="s">
-        <v>31</v>
+        <v>46</v>
       </c>
       <c r="D8" t="s">
-        <v>11</v>
+        <v>44</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>38</v>
+        <v>28</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="G8" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="H8" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B9" t="s">
         <v>9</v>
       </c>
+      <c r="C9" t="s">
+        <v>46</v>
+      </c>
       <c r="D9" t="s">
-        <v>21</v>
+        <v>40</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>33</v>
+        <v>23</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="G9" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="H9" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B10" t="s">
         <v>9</v>
       </c>
       <c r="C10" t="s">
-        <v>21</v>
+        <v>46</v>
       </c>
       <c r="D10" t="s">
-        <v>11</v>
+        <v>45</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>39</v>
+        <v>29</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>48</v>
+        <v>38</v>
       </c>
       <c r="G10" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="H10" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B11" t="s">
         <v>9</v>
       </c>
       <c r="C11" t="s">
-        <v>26</v>
+        <v>46</v>
       </c>
       <c r="D11" t="s">
-        <v>29</v>
+        <v>50</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>49</v>
+        <v>39</v>
       </c>
       <c r="G11" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="H11" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>